<commit_message>
check point3 - rate control
</commit_message>
<xml_diff>
--- a/Logs/test_esc_log.xlsx
+++ b/Logs/test_esc_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\GitHub\Drone-RTOS\Logs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA8BC041-D758-4A5A-913F-8CDE5F92C921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C5B3CCA-F240-445F-9588-A7D42F9BCE47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="828" yWindow="-108" windowWidth="22320" windowHeight="13176" xr2:uid="{B1A21DE6-F0C3-4387-996B-15DCA4957634}"/>
   </bookViews>
@@ -39,15 +39,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="9">
   <si>
     <t>Trọng lượng (g)</t>
   </si>
   <si>
     <t>PWM</t>
-  </si>
-  <si>
-    <t>MAX</t>
   </si>
   <si>
     <t>ESC_1</t>
@@ -63,6 +60,12 @@
   </si>
   <si>
     <t>ESC_3</t>
+  </si>
+  <si>
+    <t>Lực nâng (mN)</t>
+  </si>
+  <si>
+    <t>PWM pulse width (us)</t>
   </si>
 </sst>
 </file>
@@ -92,7 +95,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -115,15 +118,42 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -139,6 +169,2025 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.55631233595800522"/>
+          <c:y val="0"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="power"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$A$71:$A$90</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>67</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>102</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>145</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>273</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>315</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>360</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>402</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>385</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>401</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>401</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>401</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>401</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>401</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>401</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>401</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>401</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>401</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$B$71:$B$90</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>1110</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1150</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1200</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1250</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1300</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1350</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1400</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1450</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1500</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1530</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1580</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1630</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1680</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1730</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1780</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1830</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1880</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1930</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1980</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2030</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9B52-42C1-AB56-42656AB365E0}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1613542656"/>
+        <c:axId val="1613533536"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1613542656"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1613533536"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1613533536"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1613542656"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.2147338145231846"/>
+                  <c:y val="5.0509259259259261E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$B$2:$B$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>1110</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1150</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1200</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1250</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1300</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1350</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1400</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1450</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1500</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1560</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$C$2:$C$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>353.16</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>657.27</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1000.62</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1422.45</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1962</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2678.13</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3090.15</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3531.6000000000004</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4218.3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-8A3E-422B-BE69-1AC2232B08B8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1713126576"/>
+        <c:axId val="1713130896"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1713126576"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1713130896"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1713130896"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1713126576"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>27559</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>84786</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>332359</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>126349</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{909DC2E3-FFC3-FAB4-91E0-8BFE18283FF5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>19878</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>182217</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>324678</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>142460</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CEDB7591-E433-FE2F-90ED-A5F5FAF4810D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -463,14 +2512,21 @@
   <cols>
     <col min="1" max="1" width="36.44140625" customWidth="1"/>
     <col min="2" max="2" width="45.5546875" customWidth="1"/>
+    <col min="3" max="3" width="44.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
+      <c r="B1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1">
+        <v>9.81</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -480,8 +2536,12 @@
       <c r="B2" s="1">
         <v>1110</v>
       </c>
+      <c r="C2" s="1">
+        <f xml:space="preserve"> A2*$D$1</f>
+        <v>0</v>
+      </c>
       <c r="F2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -491,6 +2551,10 @@
       <c r="B3" s="1">
         <v>1150</v>
       </c>
+      <c r="C3" s="1">
+        <f xml:space="preserve"> A3*$D$1</f>
+        <v>353.16</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
@@ -499,6 +2563,10 @@
       <c r="B4" s="1">
         <v>1200</v>
       </c>
+      <c r="C4" s="1">
+        <f t="shared" ref="C3:C11" si="0" xml:space="preserve"> A4*$D$1</f>
+        <v>657.27</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
@@ -507,6 +2575,10 @@
       <c r="B5" s="1">
         <v>1250</v>
       </c>
+      <c r="C5" s="1">
+        <f t="shared" si="0"/>
+        <v>1000.62</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
@@ -515,6 +2587,10 @@
       <c r="B6" s="1">
         <v>1300</v>
       </c>
+      <c r="C6" s="1">
+        <f t="shared" si="0"/>
+        <v>1422.45</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
@@ -523,6 +2599,10 @@
       <c r="B7" s="1">
         <v>1350</v>
       </c>
+      <c r="C7" s="1">
+        <f t="shared" si="0"/>
+        <v>1962</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
@@ -531,6 +2611,10 @@
       <c r="B8" s="1">
         <v>1400</v>
       </c>
+      <c r="C8" s="1">
+        <f t="shared" si="0"/>
+        <v>2678.13</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
@@ -540,14 +2624,22 @@
         <f xml:space="preserve"> B8+50</f>
         <v>1450</v>
       </c>
+      <c r="C9" s="1">
+        <f t="shared" si="0"/>
+        <v>3090.15</v>
+      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>360</v>
       </c>
       <c r="B10" s="1">
-        <f t="shared" ref="B10:B21" si="0" xml:space="preserve"> B9+50</f>
+        <f t="shared" ref="B10:B21" si="1" xml:space="preserve"> B9+50</f>
         <v>1500</v>
+      </c>
+      <c r="C10" s="1">
+        <f t="shared" si="0"/>
+        <v>3531.6000000000004</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -557,103 +2649,74 @@
       <c r="B11" s="2">
         <v>1560</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>2</v>
+      <c r="C11" s="2">
+        <f t="shared" si="0"/>
+        <v>4218.3</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
-        <v>417</v>
-      </c>
-      <c r="B12" s="1">
-        <f t="shared" si="0"/>
-        <v>1610</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="B12" s="4"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
-        <v>401</v>
-      </c>
-      <c r="B13" s="1">
-        <f t="shared" si="0"/>
-        <v>1660</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="B13" s="4"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
-        <v>401</v>
-      </c>
-      <c r="B14" s="1">
-        <f t="shared" si="0"/>
-        <v>1710</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="B14" s="4"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
-        <v>401</v>
-      </c>
-      <c r="B15" s="1">
-        <f t="shared" si="0"/>
-        <v>1760</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="B15" s="4"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
-        <v>401</v>
-      </c>
-      <c r="B16" s="1">
-        <f t="shared" si="0"/>
-        <v>1810</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="B16" s="4"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
-        <v>401</v>
-      </c>
-      <c r="B17" s="1">
-        <f t="shared" si="0"/>
-        <v>1860</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="B17" s="4"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
-        <v>401</v>
-      </c>
-      <c r="B18" s="1">
-        <f t="shared" si="0"/>
-        <v>1910</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="B18" s="4"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
-        <v>401</v>
-      </c>
-      <c r="B19" s="1">
-        <f t="shared" si="0"/>
-        <v>1960</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="B19" s="4"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
-        <v>401</v>
-      </c>
-      <c r="B20" s="1">
-        <f t="shared" si="0"/>
-        <v>2010</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="B20" s="4"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
-        <v>401</v>
-      </c>
-      <c r="B21" s="1">
-        <f t="shared" si="0"/>
-        <v>2060</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="B21" s="4"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
@@ -734,7 +2797,7 @@
         <v>360</v>
       </c>
       <c r="B33" s="1">
-        <f t="shared" ref="B33" si="1" xml:space="preserve"> B32+50</f>
+        <f t="shared" ref="B33" si="2" xml:space="preserve"> B32+50</f>
         <v>1500</v>
       </c>
     </row>
@@ -751,7 +2814,7 @@
         <v>417</v>
       </c>
       <c r="B35" s="1">
-        <f t="shared" ref="B35:B44" si="2" xml:space="preserve"> B34+50</f>
+        <f t="shared" ref="B35:B44" si="3" xml:space="preserve"> B34+50</f>
         <v>1610</v>
       </c>
     </row>
@@ -760,7 +2823,7 @@
         <v>401</v>
       </c>
       <c r="B36" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1660</v>
       </c>
     </row>
@@ -769,7 +2832,7 @@
         <v>401</v>
       </c>
       <c r="B37" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1710</v>
       </c>
     </row>
@@ -778,7 +2841,7 @@
         <v>401</v>
       </c>
       <c r="B38" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1760</v>
       </c>
     </row>
@@ -787,7 +2850,7 @@
         <v>401</v>
       </c>
       <c r="B39" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1810</v>
       </c>
     </row>
@@ -796,7 +2859,7 @@
         <v>401</v>
       </c>
       <c r="B40" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1860</v>
       </c>
     </row>
@@ -805,7 +2868,7 @@
         <v>401</v>
       </c>
       <c r="B41" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1910</v>
       </c>
     </row>
@@ -814,7 +2877,7 @@
         <v>401</v>
       </c>
       <c r="B42" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1960</v>
       </c>
     </row>
@@ -823,7 +2886,7 @@
         <v>401</v>
       </c>
       <c r="B43" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2010</v>
       </c>
     </row>
@@ -832,13 +2895,13 @@
         <v>401</v>
       </c>
       <c r="B44" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2060</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
@@ -919,7 +2982,7 @@
         <v>360</v>
       </c>
       <c r="B56" s="1">
-        <f t="shared" ref="B56" si="3" xml:space="preserve"> B55+50</f>
+        <f t="shared" ref="B56" si="4" xml:space="preserve"> B55+50</f>
         <v>1500</v>
       </c>
     </row>
@@ -936,7 +2999,7 @@
         <v>417</v>
       </c>
       <c r="B58" s="1">
-        <f t="shared" ref="B58:B67" si="4" xml:space="preserve"> B57+50</f>
+        <f t="shared" ref="B58:B67" si="5" xml:space="preserve"> B57+50</f>
         <v>1610</v>
       </c>
     </row>
@@ -945,7 +3008,7 @@
         <v>401</v>
       </c>
       <c r="B59" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1660</v>
       </c>
     </row>
@@ -954,7 +3017,7 @@
         <v>401</v>
       </c>
       <c r="B60" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1710</v>
       </c>
     </row>
@@ -963,7 +3026,7 @@
         <v>401</v>
       </c>
       <c r="B61" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1760</v>
       </c>
     </row>
@@ -972,7 +3035,7 @@
         <v>401</v>
       </c>
       <c r="B62" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1810</v>
       </c>
     </row>
@@ -981,7 +3044,7 @@
         <v>401</v>
       </c>
       <c r="B63" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1860</v>
       </c>
     </row>
@@ -990,7 +3053,7 @@
         <v>401</v>
       </c>
       <c r="B64" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1910</v>
       </c>
     </row>
@@ -999,7 +3062,7 @@
         <v>401</v>
       </c>
       <c r="B65" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1960</v>
       </c>
     </row>
@@ -1008,7 +3071,7 @@
         <v>401</v>
       </c>
       <c r="B66" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>2010</v>
       </c>
     </row>
@@ -1017,13 +3080,13 @@
         <v>401</v>
       </c>
       <c r="B67" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>2060</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
@@ -1104,7 +3167,7 @@
         <v>360</v>
       </c>
       <c r="B79" s="1">
-        <f t="shared" ref="B79" si="5" xml:space="preserve"> B78+50</f>
+        <f t="shared" ref="B79" si="6" xml:space="preserve"> B78+50</f>
         <v>1500</v>
       </c>
     </row>
@@ -1121,7 +3184,7 @@
         <v>385</v>
       </c>
       <c r="B81" s="1">
-        <f t="shared" ref="B81:B90" si="6" xml:space="preserve"> B80+50</f>
+        <f t="shared" ref="B81:B90" si="7" xml:space="preserve"> B80+50</f>
         <v>1580</v>
       </c>
     </row>
@@ -1130,7 +3193,7 @@
         <v>401</v>
       </c>
       <c r="B82" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1630</v>
       </c>
     </row>
@@ -1139,7 +3202,7 @@
         <v>401</v>
       </c>
       <c r="B83" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1680</v>
       </c>
     </row>
@@ -1148,7 +3211,7 @@
         <v>401</v>
       </c>
       <c r="B84" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1730</v>
       </c>
     </row>
@@ -1157,7 +3220,7 @@
         <v>401</v>
       </c>
       <c r="B85" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1780</v>
       </c>
     </row>
@@ -1166,7 +3229,7 @@
         <v>401</v>
       </c>
       <c r="B86" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1830</v>
       </c>
     </row>
@@ -1175,7 +3238,7 @@
         <v>401</v>
       </c>
       <c r="B87" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1880</v>
       </c>
     </row>
@@ -1184,7 +3247,7 @@
         <v>401</v>
       </c>
       <c r="B88" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1930</v>
       </c>
     </row>
@@ -1193,7 +3256,7 @@
         <v>401</v>
       </c>
       <c r="B89" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1980</v>
       </c>
     </row>
@@ -1202,16 +3265,17 @@
         <v>401</v>
       </c>
       <c r="B90" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>2030</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>